<commit_message>
Samsung qty: second pass adds 24 titles
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Samsung_qty_H1_tags.xlsx
+++ b/Samsung_qty_H1_tags.xlsx
@@ -514,7 +514,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -658,41 +658,45 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>AH81-15059A</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>ah81-15059a</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="n"/>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Adaptor– Samsung Parts Usa - AH81-15059A</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Site title: samsung AH81-15059A ADAPTOR– Samsung Parts USA | Adaptor (samsungpartsusa.com)</t>
         </is>
       </c>
     </row>
@@ -768,7 +772,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -844,7 +848,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -878,7 +882,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -912,7 +916,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -946,7 +950,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1026,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1060,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>mentioned only in a collection-page summary as soundbar rear-left speaker assy $360.95; no exact product link returned; retry not done (budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1094,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>mentioned only in collection-page summary as laptop CPU heat sink $55.95; no exact product link returned; retry not done (budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1166,7 +1170,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1246,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>mentioned only in collection-page summary as soundbar Svc Jdm Screw $5.95; no exact product link returned; retry not done (budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1280,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1314,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1344,7 +1348,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1424,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1454,7 +1458,7 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1492,7 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1610,7 @@
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in samsungparts.com-filtered search; fallback retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1640,7 +1644,7 @@
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1674,7 +1678,7 @@
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1763,36 +1767,40 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>BA96-08370A</t>
         </is>
       </c>
-      <c r="C37" s="2" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>ba96-08370a</t>
         </is>
       </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="n"/>
-      <c r="F37" s="2" t="n"/>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>searched, no exact hit</t>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Laptop LCD Subins– Samsung Parts Usa Assembly - BA96-08370A</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung BA96-08370A ASSEMBLY LCD SUBINS– Samsung Parts USA | laptop LCD sub-assembly</t>
         </is>
       </c>
     </row>
@@ -1868,7 +1876,7 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1902,7 +1910,7 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1936,7 +1944,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -1983,70 +1991,78 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
         <is>
           <t>BN39-01011E</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C43" s="3" t="inlineStr">
         <is>
           <t>bn39-01011e</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="n"/>
-      <c r="F43" s="2" t="n"/>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H43" s="2" t="inlineStr">
-        <is>
-          <t>searched, no exact hit</t>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="n"/>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Lan Cable– Samsung Parts Usa - BN39-01011E</t>
+        </is>
+      </c>
+      <c r="G43" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Site title: BN39-01011E Lan Cable– Samsung Parts USA | LAN cable for select Samsung TVs</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
         <is>
           <t>AH85-01078A</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C44" s="3" t="inlineStr">
         <is>
           <t>ah85-01078a</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="n"/>
-      <c r="F44" s="2" t="n"/>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
-        <is>
-          <t>searched, no exact hit</t>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="n"/>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Oem Assembly Na-Smps Power Boa– Samsung Parts Usa - AH85-01078A</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung AH85-01078A Oem Assembly Na-Smps Power Boa– Samsung Parts USA | NA-SMPS power board assembly</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2180,7 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -2282,7 +2298,7 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -2400,41 +2416,45 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>BA83-01561A</t>
         </is>
       </c>
-      <c r="C54" s="2" t="inlineStr">
+      <c r="C54" s="3" t="inlineStr">
         <is>
           <t>ba83-01561a</t>
         </is>
       </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="n"/>
-      <c r="F54" s="2" t="n"/>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
-        <is>
-          <t>searched, no exact hit</t>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="n"/>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Jdm-Screw-Machine– Samsung Parts Usa - BA83-01561A</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>Site title: samsung BA83-01561A JDM-SCREW-MACHINE– Samsung Parts USA | JDM screw machine; fits select Samsung laptops</t>
         </is>
       </c>
     </row>
@@ -2510,7 +2530,7 @@
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -2586,7 +2606,7 @@
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2640,7 @@
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -2696,7 +2716,7 @@
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -2730,7 +2750,7 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -2764,7 +2784,7 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -2924,7 +2944,7 @@
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -2958,7 +2978,7 @@
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -3034,7 +3054,7 @@
       </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -3068,7 +3088,7 @@
       </c>
       <c r="H71" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -3144,7 +3164,7 @@
       </c>
       <c r="H73" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -3178,41 +3198,45 @@
       </c>
       <c r="H74" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
         <is>
           <t>BA96-08319B</t>
         </is>
       </c>
-      <c r="C75" s="2" t="inlineStr">
+      <c r="C75" s="3" t="inlineStr">
         <is>
           <t>ba96-08319b</t>
         </is>
       </c>
-      <c r="D75" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E75" s="2" t="n"/>
-      <c r="F75" s="2" t="n"/>
-      <c r="G75" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H75" s="2" t="inlineStr">
-        <is>
-          <t>searched, no exact hit</t>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="n"/>
+      <c r="F75" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Laptop LCD Subins-Silver– Samsung Parts Usa Assembly - BA96-08319B</t>
+        </is>
+      </c>
+      <c r="G75" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H75" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung BA96-08319B ASSEMBLY LCD SUBINS-SILVER– Samsung Parts USA | laptop LCD assembly (subins, silver)</t>
         </is>
       </c>
     </row>
@@ -3246,7 +3270,7 @@
       </c>
       <c r="H76" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -3322,7 +3346,7 @@
       </c>
       <c r="H78" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -3440,7 +3464,7 @@
       </c>
       <c r="H81" s="2" t="inlineStr">
         <is>
-          <t>only sibling BA98-03666B found; retry found nothing</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -3655,36 +3679,40 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B87" s="2" t="inlineStr">
+      <c r="A87" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B87" s="3" t="inlineStr">
         <is>
           <t>AH91-09033F</t>
         </is>
       </c>
-      <c r="C87" s="2" t="inlineStr">
+      <c r="C87" s="3" t="inlineStr">
         <is>
           <t>ah91-09033f</t>
         </is>
       </c>
-      <c r="D87" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="n"/>
-      <c r="F87" s="2" t="n"/>
-      <c r="G87" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H87" s="2" t="inlineStr">
-        <is>
-          <t>retry found nothing</t>
+      <c r="D87" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E87" s="3" t="n"/>
+      <c r="F87" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Speaker Assembly - AH91-09033F</t>
+        </is>
+      </c>
+      <c r="G87" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H87" s="3" t="inlineStr">
+        <is>
+          <t>Site title: AH91-09033F ASSEMBLY SPEAKER | Assembly speaker (soundbar/TV speaker); page notes no longer available with comparable replacement</t>
         </is>
       </c>
     </row>
@@ -3718,7 +3746,7 @@
       </c>
       <c r="H88" s="2" t="inlineStr">
         <is>
-          <t>retry found nothing</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -3794,7 +3822,7 @@
       </c>
       <c r="H90" s="2" t="inlineStr">
         <is>
-          <t>only sibling AH94-03880A found; retry found nothing</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -3828,7 +3856,7 @@
       </c>
       <c r="H91" s="2" t="inlineStr">
         <is>
-          <t>retry found nothing</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4134,7 @@
       </c>
       <c r="H98" s="2" t="inlineStr">
         <is>
-          <t>retry found nothing</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -4220,41 +4248,45 @@
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B102" s="2" t="inlineStr">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
         <is>
           <t>BA98-01478A</t>
         </is>
       </c>
-      <c r="C102" s="2" t="inlineStr">
+      <c r="C102" s="3" t="inlineStr">
         <is>
           <t>ba98-01478a</t>
         </is>
       </c>
-      <c r="D102" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E102" s="2" t="n"/>
-      <c r="F102" s="2" t="n"/>
-      <c r="G102" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H102" s="2" t="inlineStr">
-        <is>
-          <t>searched, no exact hit</t>
+      <c r="D102" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E102" s="3" t="n"/>
+      <c r="F102" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Case-Lower Lcd– Samsung Parts Usa Assembly - BA98-01478A</t>
+        </is>
+      </c>
+      <c r="G102" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H102" s="3" t="inlineStr">
+        <is>
+          <t>Site title: BA98-01478A ASSEMBLY CASE-LOWER LCD– Samsung Parts USA | laptop lower LCD case assembly</t>
         </is>
       </c>
     </row>
@@ -4372,7 +4404,7 @@
       </c>
       <c r="H105" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -4406,7 +4438,7 @@
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4514,7 @@
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -4516,41 +4548,45 @@
       </c>
       <c r="H109" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B110" s="2" t="inlineStr">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
         <is>
           <t>AH81-15944A</t>
         </is>
       </c>
-      <c r="C110" s="2" t="inlineStr">
+      <c r="C110" s="3" t="inlineStr">
         <is>
           <t>ah81-15944a</t>
         </is>
       </c>
-      <c r="D110" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E110" s="2" t="n"/>
-      <c r="F110" s="2" t="n"/>
-      <c r="G110" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H110" s="2" t="inlineStr">
-        <is>
-          <t>searched, no exact hit</t>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E110" s="3" t="n"/>
+      <c r="F110" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Service Jdm-Remocon– Samsung Parts Usa - AH81-15944A</t>
+        </is>
+      </c>
+      <c r="G110" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H110" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung AH81-15944A Service Jdm-Remocon– Samsung Parts USA | remote control (Service JDM-Remocon) for speakers/soundbars</t>
         </is>
       </c>
     </row>
@@ -4584,7 +4620,7 @@
       </c>
       <c r="H111" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -4618,7 +4654,7 @@
       </c>
       <c r="H112" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -4652,7 +4688,7 @@
       </c>
       <c r="H113" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -4728,41 +4764,45 @@
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B116" s="2" t="inlineStr">
+      <c r="A116" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
         <is>
           <t>AH81-15682A</t>
         </is>
       </c>
-      <c r="C116" s="2" t="inlineStr">
+      <c r="C116" s="3" t="inlineStr">
         <is>
           <t>ah81-15682a</t>
         </is>
       </c>
-      <c r="D116" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E116" s="2" t="n"/>
-      <c r="F116" s="2" t="n"/>
-      <c r="G116" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H116" s="2" t="inlineStr">
-        <is>
-          <t>searched, no exact hit</t>
+      <c r="D116" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E116" s="3" t="n"/>
+      <c r="F116" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Samsung Service Jdm-Sub W/F Ps-Wr45Bb|Samsung Parts Usa - AH81-15682A</t>
+        </is>
+      </c>
+      <c r="G116" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H116" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung samsung AH81-15682A SERVICE JDM-SUB W/F PS-WR45BB|Samsung Parts USA | service JDM sub woofer PS-WR45BB; speaker/soundbar; listed no longer available</t>
         </is>
       </c>
     </row>
@@ -4796,7 +4836,7 @@
       </c>
       <c r="H117" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -4830,7 +4870,7 @@
       </c>
       <c r="H118" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4904,7 @@
       </c>
       <c r="H119" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -4898,7 +4938,7 @@
       </c>
       <c r="H120" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -4932,7 +4972,7 @@
       </c>
       <c r="H121" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -4966,7 +5006,7 @@
       </c>
       <c r="H122" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -5042,7 +5082,7 @@
       </c>
       <c r="H124" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5116,7 @@
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -5110,7 +5150,7 @@
       </c>
       <c r="H126" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -5144,7 +5184,7 @@
       </c>
       <c r="H127" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -5178,7 +5218,7 @@
       </c>
       <c r="H128" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -5212,7 +5252,7 @@
       </c>
       <c r="H129" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -5246,7 +5286,7 @@
       </c>
       <c r="H130" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -5280,7 +5320,7 @@
       </c>
       <c r="H131" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -5411,36 +5451,44 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B135" s="2" t="inlineStr">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
         <is>
           <t>BA98-03038A</t>
         </is>
       </c>
-      <c r="C135" s="2" t="inlineStr">
+      <c r="C135" t="inlineStr">
         <is>
           <t>ba98-03038a</t>
         </is>
       </c>
-      <c r="D135" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E135" s="2" t="n"/>
-      <c r="F135" s="2" t="n"/>
-      <c r="G135" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H135" s="2" t="inlineStr">
-        <is>
-          <t>searched, no exact hit</t>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Verified (page found)</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>https://samsungparts.com/products/ba98-03038a</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Rubber Foot Down Assembly - BA98-03038A</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Site title: Samsung BA98-03038A ASSEMBLY RUBBER FOOT DOWN | laptop assembly rubber foot down</t>
         </is>
       </c>
     </row>
@@ -5474,7 +5522,7 @@
       </c>
       <c r="H136" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -5634,7 +5682,7 @@
       </c>
       <c r="H140" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -5794,7 +5842,7 @@
       </c>
       <c r="H144" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -5912,7 +5960,7 @@
       </c>
       <c r="H147" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -5959,36 +6007,44 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B149" s="2" t="inlineStr">
+      <c r="A149" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
         <is>
           <t>6001-002610</t>
         </is>
       </c>
-      <c r="C149" s="2" t="inlineStr">
+      <c r="C149" s="3" t="inlineStr">
         <is>
           <t>6001-002610</t>
         </is>
       </c>
-      <c r="D149" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E149" s="2" t="n"/>
-      <c r="F149" s="2" t="n"/>
-      <c r="G149" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H149" s="2" t="inlineStr">
-        <is>
-          <t>searched, no exact hit</t>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>Verified (page found)</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>https://samsungparts.com/products/6001-002610</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Machine Screw - 6001-002610</t>
+        </is>
+      </c>
+      <c r="G149" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H149" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung 6001-002610 Screw-Machine | machine screw</t>
         </is>
       </c>
     </row>
@@ -6148,7 +6204,7 @@
       </c>
       <c r="H153" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -6182,7 +6238,7 @@
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -6216,7 +6272,7 @@
       </c>
       <c r="H155" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -6250,7 +6306,7 @@
       </c>
       <c r="H156" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -6326,41 +6382,45 @@
       </c>
       <c r="H158" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B159" s="2" t="inlineStr">
+      <c r="A159" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B159" s="3" t="inlineStr">
         <is>
           <t>AH81-13316A</t>
         </is>
       </c>
-      <c r="C159" s="2" t="inlineStr">
+      <c r="C159" s="3" t="inlineStr">
         <is>
           <t>ah81-13316a</t>
         </is>
       </c>
-      <c r="D159" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E159" s="2" t="n"/>
-      <c r="F159" s="2" t="n"/>
-      <c r="G159" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H159" s="2" t="inlineStr">
-        <is>
-          <t>searched, no exact hit</t>
+      <c r="D159" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E159" s="3" t="n"/>
+      <c r="F159" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Service Jdm Antenna|Samsung Parts Usa - AH81-13316A</t>
+        </is>
+      </c>
+      <c r="G159" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H159" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung AH81-13316A Svc Jdm Antenna|Samsung Parts USA | Svc Jdm Antenna</t>
         </is>
       </c>
     </row>
@@ -6520,7 +6580,7 @@
       </c>
       <c r="H163" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on first search or retry (neighbouring numbers only)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -6672,7 +6732,7 @@
       </c>
       <c r="H167" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on first search or retry (neighbouring numbers only)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -6786,7 +6846,7 @@
       </c>
       <c r="H170" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on first search or retry (neighbouring numbers only)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -6820,41 +6880,45 @@
       </c>
       <c r="H171" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on first search or retry (neighbouring numbers only)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
     <row r="172">
-      <c r="A172" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B172" s="2" t="inlineStr">
+      <c r="A172" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
         <is>
           <t>BA97-12306A</t>
         </is>
       </c>
-      <c r="C172" s="2" t="inlineStr">
+      <c r="C172" s="3" t="inlineStr">
         <is>
           <t>ba97-12306a</t>
         </is>
       </c>
-      <c r="D172" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E172" s="2" t="n"/>
-      <c r="F172" s="2" t="n"/>
-      <c r="G172" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H172" s="2" t="inlineStr">
-        <is>
-          <t>no exact hit on first search or retry (neighbouring numbers only)</t>
+      <c r="D172" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E172" s="3" t="n"/>
+      <c r="F172" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Assembly Case Front-Top– Samsung Parts Usa - BA97-12306A</t>
+        </is>
+      </c>
+      <c r="G172" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H172" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung BA97-12306A Assy Case Front-Top– Samsung Parts USA | Assy Case Front-Top (laptop case)</t>
         </is>
       </c>
     </row>
@@ -6930,7 +6994,7 @@
       </c>
       <c r="H174" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on first search or retry (neighbouring numbers only)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -6964,7 +7028,7 @@
       </c>
       <c r="H175" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on first search or retry (neighbouring numbers only)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -7221,36 +7285,40 @@
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B182" s="2" t="inlineStr">
+      <c r="A182" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B182" s="3" t="inlineStr">
         <is>
           <t>BA98-03232B</t>
         </is>
       </c>
-      <c r="C182" s="2" t="inlineStr">
+      <c r="C182" s="3" t="inlineStr">
         <is>
           <t>ba98-03232b</t>
         </is>
       </c>
-      <c r="D182" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E182" s="2" t="n"/>
-      <c r="F182" s="2" t="n"/>
-      <c r="G182" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H182" s="2" t="inlineStr">
-        <is>
-          <t>INCOMPLETE: first domain search had no exact hit; retry NOT run (web search budget exhausted)</t>
+      <c r="D182" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E182" s="3" t="n"/>
+      <c r="F182" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Case Rear|Samsung Parts Usa Assembly - BA98-03232B</t>
+        </is>
+      </c>
+      <c r="G182" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H182" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung BA98-03232B ASSEMBLY CASE REAR|Samsung Parts USA | Assembly case rear (laptop); page notes no longer available with comparable replacement</t>
         </is>
       </c>
     </row>
@@ -7284,7 +7352,7 @@
       </c>
       <c r="H183" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE: first domain search had no exact hit; retry NOT run (web search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -7318,7 +7386,7 @@
       </c>
       <c r="H184" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE: first domain search had no exact hit; retry NOT run (web search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -7352,7 +7420,7 @@
       </c>
       <c r="H185" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE: first domain search had no exact hit; retry NOT run (web search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -7428,7 +7496,7 @@
       </c>
       <c r="H187" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE: first domain search had no exact hit; retry NOT run (web search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -7504,7 +7572,7 @@
       </c>
       <c r="H189" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE: first domain search had no exact hit; retry NOT run (web search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -7538,7 +7606,7 @@
       </c>
       <c r="H190" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -7572,7 +7640,7 @@
       </c>
       <c r="H191" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -7606,7 +7674,7 @@
       </c>
       <c r="H192" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -7640,7 +7708,7 @@
       </c>
       <c r="H193" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -7674,7 +7742,7 @@
       </c>
       <c r="H194" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -7708,7 +7776,7 @@
       </c>
       <c r="H195" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -7784,7 +7852,7 @@
       </c>
       <c r="H197" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -7902,7 +7970,7 @@
       </c>
       <c r="H200" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -7978,7 +8046,7 @@
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -8012,7 +8080,7 @@
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -8059,36 +8127,40 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B205" s="2" t="inlineStr">
+      <c r="A205" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
         <is>
           <t>6001-002653</t>
         </is>
       </c>
-      <c r="C205" s="2" t="inlineStr">
+      <c r="C205" s="3" t="inlineStr">
         <is>
           <t>6001-002653</t>
         </is>
       </c>
-      <c r="D205" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E205" s="2" t="n"/>
-      <c r="F205" s="2" t="n"/>
-      <c r="G205" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H205" s="2" t="inlineStr">
-        <is>
-          <t>searched, no exact hit</t>
+      <c r="D205" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E205" s="3" t="n"/>
+      <c r="F205" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Screw, M3 X 6– Samsung Parts Usa - 6001-002653</t>
+        </is>
+      </c>
+      <c r="G205" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H205" s="3" t="inlineStr">
+        <is>
+          <t>Site title: 6001-002653 Screw, M3 x 6– Samsung Parts USA | M3 x 6 screw</t>
         </is>
       </c>
     </row>
@@ -8122,7 +8194,7 @@
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -8240,7 +8312,7 @@
       </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -8274,7 +8346,7 @@
       </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -8350,7 +8422,7 @@
       </c>
       <c r="H212" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -8426,7 +8498,7 @@
       </c>
       <c r="H214" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -8502,7 +8574,7 @@
       </c>
       <c r="H216" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -8536,7 +8608,7 @@
       </c>
       <c r="H217" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -8654,7 +8726,7 @@
       </c>
       <c r="H220" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -8688,7 +8760,7 @@
       </c>
       <c r="H221" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -8722,7 +8794,7 @@
       </c>
       <c r="H222" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -8756,7 +8828,7 @@
       </c>
       <c r="H223" s="2" t="inlineStr">
         <is>
-          <t>searched, no exact hit</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -9332,7 +9404,7 @@
       </c>
       <c r="H239" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -9450,7 +9522,7 @@
       </c>
       <c r="H242" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -9484,7 +9556,7 @@
       </c>
       <c r="H243" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -9518,7 +9590,7 @@
       </c>
       <c r="H244" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -9552,7 +9624,7 @@
       </c>
       <c r="H245" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -9641,36 +9713,44 @@
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B248" s="2" t="inlineStr">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
         <is>
           <t>BN39-01652V</t>
         </is>
       </c>
-      <c r="C248" s="2" t="inlineStr">
+      <c r="C248" t="inlineStr">
         <is>
           <t>bn39-01652v</t>
         </is>
       </c>
-      <c r="D248" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E248" s="2" t="n"/>
-      <c r="F248" s="2" t="n"/>
-      <c r="G248" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H248" s="2" t="inlineStr">
-        <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Verified (page found)</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>https://samsungparts.com/products/bn39-01652v</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>Samsung TV Lead Connector - BN39-01652V</t>
+        </is>
+      </c>
+      <c r="G248" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H248" t="inlineStr">
+        <is>
+          <t>Site title: Samsung BN39-01652V Lead Connector | Lead connector for LED TVs; listed no longer available, comparable part suggested</t>
         </is>
       </c>
     </row>
@@ -9704,7 +9784,7 @@
       </c>
       <c r="H249" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -9738,7 +9818,7 @@
       </c>
       <c r="H250" s="2" t="inlineStr">
         <is>
-          <t>search summary mentioned a battery assembly listing but no link URL returned; retry not done</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -9772,7 +9852,7 @@
       </c>
       <c r="H251" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -9861,36 +9941,40 @@
       </c>
     </row>
     <row r="254">
-      <c r="A254" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B254" s="2" t="inlineStr">
+      <c r="A254" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B254" s="3" t="inlineStr">
         <is>
           <t>3404-001490</t>
         </is>
       </c>
-      <c r="C254" s="2" t="inlineStr">
+      <c r="C254" s="3" t="inlineStr">
         <is>
           <t>3404-001490</t>
         </is>
       </c>
-      <c r="D254" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E254" s="2" t="n"/>
-      <c r="F254" s="2" t="n"/>
-      <c r="G254" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H254" s="2" t="inlineStr">
-        <is>
-          <t>search summary mentioned Switch-Tact listing but no link URL returned; retry not done</t>
+      <c r="D254" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E254" s="3" t="n"/>
+      <c r="F254" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Vacuum Switch-Tact– Samsung Parts Usa - 3404-001490</t>
+        </is>
+      </c>
+      <c r="G254" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H254" s="3" t="inlineStr">
+        <is>
+          <t>Site title: 3404-001490 SWITCH-TACT– Samsung Parts USA | Switch-Tact; listed under television parts (page text also mentions vacuum cleaner models)</t>
         </is>
       </c>
     </row>
@@ -9924,7 +10008,7 @@
       </c>
       <c r="H255" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -9958,7 +10042,7 @@
       </c>
       <c r="H256" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -9992,41 +10076,45 @@
       </c>
       <c r="H257" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
     <row r="258">
-      <c r="A258" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B258" s="2" t="inlineStr">
+      <c r="A258" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B258" s="3" t="inlineStr">
         <is>
           <t>BN39-02207C</t>
         </is>
       </c>
-      <c r="C258" s="2" t="inlineStr">
+      <c r="C258" s="3" t="inlineStr">
         <is>
           <t>bn39-02207c</t>
         </is>
       </c>
-      <c r="D258" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E258" s="2" t="n"/>
-      <c r="F258" s="2" t="n"/>
-      <c r="G258" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H258" s="2" t="inlineStr">
-        <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+      <c r="D258" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E258" s="3" t="n"/>
+      <c r="F258" s="3" t="inlineStr">
+        <is>
+          <t>Samsung TV Lead Connector-Power– Samsung Parts Usa - BN39-02207C</t>
+        </is>
+      </c>
+      <c r="G258" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H258" s="3" t="inlineStr">
+        <is>
+          <t>Site title: BN39-02207C LEAD CONNECTOR-POWER– Samsung Parts USA | Lead Connector-Power (TV)</t>
         </is>
       </c>
     </row>
@@ -10060,7 +10148,7 @@
       </c>
       <c r="H259" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -10094,7 +10182,7 @@
       </c>
       <c r="H260" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -10128,7 +10216,7 @@
       </c>
       <c r="H261" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -10162,7 +10250,7 @@
       </c>
       <c r="H262" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -10196,7 +10284,7 @@
       </c>
       <c r="H263" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -10230,7 +10318,7 @@
       </c>
       <c r="H264" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -10264,7 +10352,7 @@
       </c>
       <c r="H265" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -10298,7 +10386,7 @@
       </c>
       <c r="H266" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -10332,41 +10420,49 @@
       </c>
       <c r="H267" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
     <row r="268">
-      <c r="A268" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B268" s="2" t="inlineStr">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
         <is>
           <t>BA31-00117A</t>
         </is>
       </c>
-      <c r="C268" s="2" t="inlineStr">
+      <c r="C268" t="inlineStr">
         <is>
           <t>ba31-00117a</t>
         </is>
       </c>
-      <c r="D268" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E268" s="2" t="n"/>
-      <c r="F268" s="2" t="n"/>
-      <c r="G268" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H268" s="2" t="inlineStr">
-        <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>Verified (page found)</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>https://samsungparts.com/products/ba31-00117a</t>
+        </is>
+      </c>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>Samsung Laptop CPU Fan - BA31-00117A</t>
+        </is>
+      </c>
+      <c r="G268" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H268" t="inlineStr">
+        <is>
+          <t>Site title: Samsung BA31-00117A Fan-Cpu | Laptop CPU cooling fan; listed no longer available, comparable part suggested</t>
         </is>
       </c>
     </row>
@@ -10400,7 +10496,7 @@
       </c>
       <c r="H269" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -10518,7 +10614,7 @@
       </c>
       <c r="H272" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -10552,7 +10648,7 @@
       </c>
       <c r="H273" s="2" t="inlineStr">
         <is>
-          <t>only category-page mention, no product link; retry not done</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -10586,7 +10682,7 @@
       </c>
       <c r="H274" s="2" t="inlineStr">
         <is>
-          <t>no exact hit in domain search; retry not done (search budget exhausted)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -12218,7 +12314,7 @@
       </c>
       <c r="H318" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -12252,7 +12348,7 @@
       </c>
       <c r="H319" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -12286,7 +12382,7 @@
       </c>
       <c r="H320" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -12320,7 +12416,7 @@
       </c>
       <c r="H321" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -12354,7 +12450,7 @@
       </c>
       <c r="H322" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -12388,7 +12484,7 @@
       </c>
       <c r="H323" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -12422,7 +12518,7 @@
       </c>
       <c r="H324" s="2" t="inlineStr">
         <is>
-          <t>search showed collection page 'new-collection?page=244' naming 'Samsung AH81-15342A Service Jdm-Cable-Ffc' only; no products/ URL; retry not run (budget)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -12456,41 +12552,45 @@
       </c>
       <c r="H325" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
     <row r="326">
-      <c r="A326" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B326" s="2" t="inlineStr">
+      <c r="A326" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B326" s="3" t="inlineStr">
         <is>
           <t>BA44-00298A</t>
         </is>
       </c>
-      <c r="C326" s="2" t="inlineStr">
+      <c r="C326" s="3" t="inlineStr">
         <is>
           <t>ba44-00298a</t>
         </is>
       </c>
-      <c r="D326" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E326" s="2" t="n"/>
-      <c r="F326" s="2" t="n"/>
-      <c r="G326" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H326" s="2" t="inlineStr">
-        <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+      <c r="D326" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E326" s="3" t="n"/>
+      <c r="F326" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Samsung AC Adapter|Samsung Parts Usa - BA44-00298A</t>
+        </is>
+      </c>
+      <c r="G326" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H326" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung samsung BA44-00298A AC ADAPTER|Samsung Parts USA | AC adapter for Samsung computer/laptop; listed as discontinued</t>
         </is>
       </c>
     </row>
@@ -12524,7 +12624,7 @@
       </c>
       <c r="H327" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -12558,41 +12658,45 @@
       </c>
       <c r="H328" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
     <row r="329">
-      <c r="A329" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B329" s="2" t="inlineStr">
+      <c r="A329" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B329" s="3" t="inlineStr">
         <is>
           <t>AH94-03759A</t>
         </is>
       </c>
-      <c r="C329" s="2" t="inlineStr">
+      <c r="C329" s="3" t="inlineStr">
         <is>
           <t>ah94-03759a</t>
         </is>
       </c>
-      <c r="D329" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E329" s="2" t="n"/>
-      <c r="F329" s="2" t="n"/>
-      <c r="G329" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H329" s="2" t="inlineStr">
-        <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+      <c r="D329" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E329" s="3" t="n"/>
+      <c r="F329" s="3" t="inlineStr">
+        <is>
+          <t>Samsung TV PCB Assembly|Samsung Parts Usa - AH94-03759A</t>
+        </is>
+      </c>
+      <c r="G329" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H329" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung AH94-03759A Pcb Assembly|Samsung Parts USA | PCB assembly for televisions; listed as no longer available</t>
         </is>
       </c>
     </row>
@@ -12626,41 +12730,45 @@
       </c>
       <c r="H330" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
     <row r="331">
-      <c r="A331" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B331" s="2" t="inlineStr">
+      <c r="A331" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B331" s="3" t="inlineStr">
         <is>
           <t>6001-001773</t>
         </is>
       </c>
-      <c r="C331" s="2" t="inlineStr">
+      <c r="C331" s="3" t="inlineStr">
         <is>
           <t>6001-001773</t>
         </is>
       </c>
-      <c r="D331" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E331" s="2" t="n"/>
-      <c r="F331" s="2" t="n"/>
-      <c r="G331" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H331" s="2" t="inlineStr">
-        <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+      <c r="D331" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E331" s="3" t="n"/>
+      <c r="F331" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Machine Washer Or Dryer Screw - 6001-001773</t>
+        </is>
+      </c>
+      <c r="G331" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H331" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Washer or Dryer 6001-001773 Screw-Machine | machine screw for Samsung washer/dryer</t>
         </is>
       </c>
     </row>
@@ -12778,7 +12886,7 @@
       </c>
       <c r="H334" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -12812,7 +12920,7 @@
       </c>
       <c r="H335" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -12888,7 +12996,7 @@
       </c>
       <c r="H337" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -12922,7 +13030,7 @@
       </c>
       <c r="H338" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -12956,7 +13064,7 @@
       </c>
       <c r="H339" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -12990,7 +13098,7 @@
       </c>
       <c r="H340" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -13024,7 +13132,7 @@
       </c>
       <c r="H341" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -13058,41 +13166,45 @@
       </c>
       <c r="H342" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
     <row r="343">
-      <c r="A343" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B343" s="2" t="inlineStr">
+      <c r="A343" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B343" s="3" t="inlineStr">
         <is>
           <t>BA39-01262A</t>
         </is>
       </c>
-      <c r="C343" s="2" t="inlineStr">
+      <c r="C343" s="3" t="inlineStr">
         <is>
           <t>ba39-01262a</t>
         </is>
       </c>
-      <c r="D343" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E343" s="2" t="n"/>
-      <c r="F343" s="2" t="n"/>
-      <c r="G343" s="2" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="H343" s="2" t="inlineStr">
-        <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+      <c r="D343" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E343" s="3" t="n"/>
+      <c r="F343" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Cable– Samsung Parts Usa - BA39-01262A</t>
+        </is>
+      </c>
+      <c r="G343" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H343" s="3" t="inlineStr">
+        <is>
+          <t>Site title: BA39-01262A Cable– Samsung Parts USA | cable (BA39 laptop-family); OEM part</t>
         </is>
       </c>
     </row>
@@ -13168,7 +13280,7 @@
       </c>
       <c r="H345" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -13328,7 +13440,7 @@
       </c>
       <c r="H349" s="2" t="inlineStr">
         <is>
-          <t>samsungparts sitemap xml lists https://samsungparts.com/products/bn39-02709a but no titled product link returned; not counted; retry not run (budget)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -13404,7 +13516,7 @@
       </c>
       <c r="H351" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -13480,7 +13592,7 @@
       </c>
       <c r="H353" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -13514,7 +13626,7 @@
       </c>
       <c r="H354" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -13590,7 +13702,7 @@
       </c>
       <c r="H356" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -13624,7 +13736,7 @@
       </c>
       <c r="H357" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -13658,7 +13770,7 @@
       </c>
       <c r="H358" s="2" t="inlineStr">
         <is>
-          <t>sitemap xml lists products/bn39-02919a ('Lead Connector-Power;Qn65S95Ca') but no titled product link returned; not counted; retry not run (budget)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -13734,7 +13846,7 @@
       </c>
       <c r="H360" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -13768,7 +13880,7 @@
       </c>
       <c r="H361" s="2" t="inlineStr">
         <is>
-          <t>only seen as 'Trans Switching' on dvd-player-parts collection page, no products/ URL; retry not run (budget)</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>
@@ -13802,7 +13914,7 @@
       </c>
       <c r="H362" s="2" t="inlineStr">
         <is>
-          <t>no exact hit on samsungparts.com; retry (Samsung &lt;PN&gt;) not run, search budget exhausted</t>
+          <t>pass2 searched, no exact hit</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Samsung qty: tidy open-search titles
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Samsung_qty_H1_tags.xlsx
+++ b/Samsung_qty_H1_tags.xlsx
@@ -5034,7 +5034,7 @@
       <c r="E116" s="3" t="n"/>
       <c r="F116" s="3" t="inlineStr">
         <is>
-          <t>Samsung Soundbar Samsung Service Jdm-Sub W/F Ps-Wr45Bb|Samsung Parts Usa - AH81-15682A</t>
+          <t>Samsung Soundbar Service Jdm-Sub W/F Ps-Wr45Bb - AH81-15682A</t>
         </is>
       </c>
       <c r="G116" s="3" t="inlineStr">
@@ -6748,7 +6748,7 @@
       <c r="E159" s="3" t="n"/>
       <c r="F159" s="3" t="inlineStr">
         <is>
-          <t>Samsung Service Jdm Antenna|Samsung Parts Usa - AH81-13316A</t>
+          <t>Samsung Service Jdm Antenna - AH81-13316A</t>
         </is>
       </c>
       <c r="G159" s="3" t="inlineStr">
@@ -7674,7 +7674,7 @@
       <c r="E182" s="3" t="n"/>
       <c r="F182" s="3" t="inlineStr">
         <is>
-          <t>Samsung Laptop Case Rear|Samsung Parts Usa Assembly - BA98-03232B</t>
+          <t>Samsung Laptop Case Rear Assembly - BA98-03232B</t>
         </is>
       </c>
       <c r="G182" s="3" t="inlineStr">
@@ -12002,7 +12002,7 @@
       <c r="E292" s="3" t="n"/>
       <c r="F292" s="3" t="inlineStr">
         <is>
-          <t>Samsung Laptop Case Rear|Samsung Parts Usa Assembly - BA98-02902A</t>
+          <t>Samsung Laptop Case Rear Assembly - BA98-02902A</t>
         </is>
       </c>
       <c r="G292" s="3" t="inlineStr">
@@ -12836,7 +12836,7 @@
       <c r="E313" s="3" t="n"/>
       <c r="F313" s="3" t="inlineStr">
         <is>
-          <t>Samsung Samsung Service Jdm-Power Module|Samsung Parts Usa - AH81-15334A</t>
+          <t>Samsung Power Module Service Jdm - AH81-15334A</t>
         </is>
       </c>
       <c r="G313" s="3" t="inlineStr">
@@ -13334,7 +13334,7 @@
       <c r="E326" s="3" t="n"/>
       <c r="F326" s="3" t="inlineStr">
         <is>
-          <t>Samsung Laptop Samsung AC Adapter|Samsung Parts Usa - BA44-00298A</t>
+          <t>Samsung Laptop AC Adapter - BA44-00298A</t>
         </is>
       </c>
       <c r="G326" s="3" t="inlineStr">
@@ -13448,7 +13448,7 @@
       <c r="E329" s="3" t="n"/>
       <c r="F329" s="3" t="inlineStr">
         <is>
-          <t>Samsung TV PCB Assembly|Samsung Parts Usa - AH94-03759A</t>
+          <t>Samsung TV PCB Assembly - AH94-03759A</t>
         </is>
       </c>
       <c r="G329" s="3" t="inlineStr">
@@ -19028,7 +19028,7 @@
       <c r="E471" s="3" t="n"/>
       <c r="F471" s="3" t="inlineStr">
         <is>
-          <t>Samsung Samsung OLED Board|Samsung Parts Usa - AH81-15485A</t>
+          <t>Samsung OLED Board - AH81-15485A</t>
         </is>
       </c>
       <c r="G471" s="3" t="inlineStr">
@@ -20360,7 +20360,7 @@
       <c r="E505" s="3" t="n"/>
       <c r="F505" s="3" t="inlineStr">
         <is>
-          <t>Samsung Laptop Adaptor|Samsung Parts Usa - BA44-00353A</t>
+          <t>Samsung Laptop Adaptor - BA44-00353A</t>
         </is>
       </c>
       <c r="G505" s="3" t="inlineStr">
@@ -22462,7 +22462,7 @@
       <c r="E558" s="3" t="n"/>
       <c r="F558" s="3" t="inlineStr">
         <is>
-          <t>Samsung Soundbar Bracket P-Wall|Samsung Parts Usa Assembly - AH96-03944B</t>
+          <t>Samsung Soundbar Wall Bracket P Assembly - AH96-03944B</t>
         </is>
       </c>
       <c r="G558" s="3" t="inlineStr">
@@ -22892,7 +22892,7 @@
       <c r="E569" s="3" t="n"/>
       <c r="F569" s="3" t="inlineStr">
         <is>
-          <t>Samsung Ckd-Remote Control|Samsung Parts Usa - AA83-00654A</t>
+          <t>Samsung Remote Control Ckd - AA83-00654A</t>
         </is>
       </c>
       <c r="G569" s="3" t="inlineStr">
@@ -25404,7 +25404,7 @@
       <c r="E633" s="3" t="n"/>
       <c r="F633" s="3" t="inlineStr">
         <is>
-          <t>Samsung Samsung Service Jdm-Remote Control|Samsung Parts Usa - AH81-14847A</t>
+          <t>Samsung Remote Control Service Jdm - AH81-14847A</t>
         </is>
       </c>
       <c r="G633" s="3" t="inlineStr">
@@ -26104,7 +26104,7 @@
       <c r="E651" s="3" t="n"/>
       <c r="F651" s="3" t="inlineStr">
         <is>
-          <t>Samsung Samsung Service Jdm-Power Cord|Samsung Parts Usa - AH81-14849A</t>
+          <t>Samsung Power Cord Service Jdm - AH81-14849A</t>
         </is>
       </c>
       <c r="G651" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Samsung qty: final variant-search pass adds 34 titles
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Samsung_qty_H1_tags.xlsx
+++ b/Samsung_qty_H1_tags.xlsx
@@ -29541,40 +29541,44 @@
       </c>
     </row>
     <row r="739">
-      <c r="A739" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B739" s="2" t="inlineStr">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
         <is>
           <t>BA43-00391A</t>
         </is>
       </c>
-      <c r="C739" s="2" t="inlineStr">
+      <c r="C739" t="inlineStr">
         <is>
           <t>ba43-00391a</t>
         </is>
       </c>
-      <c r="D739" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E739" s="2" t="n"/>
-      <c r="F739" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Laptop Replacement Part - BA43-00391A</t>
-        </is>
-      </c>
-      <c r="G739" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H739" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D739" t="inlineStr">
+        <is>
+          <t>Verified (page found)</t>
+        </is>
+      </c>
+      <c r="E739" t="inlineStr">
+        <is>
+          <t>https://samsungparts.com/products/ba43-00391a</t>
+        </is>
+      </c>
+      <c r="F739" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Incell Battery Pack - BA43-00391A</t>
+        </is>
+      </c>
+      <c r="G739" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H739" t="inlineStr">
+        <is>
+          <t>Site title: Samsung BA43-00391A Incell Battery Pack-P41Gcj-02- | Incell Battery Pack / fits laptop</t>
         </is>
       </c>
     </row>
@@ -30131,40 +30135,40 @@
       </c>
     </row>
     <row r="754">
-      <c r="A754" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B754" s="2" t="inlineStr">
+      <c r="A754" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B754" s="3" t="inlineStr">
         <is>
           <t>BA81-18114A</t>
         </is>
       </c>
-      <c r="C754" s="2" t="inlineStr">
+      <c r="C754" s="3" t="inlineStr">
         <is>
           <t>ba81-18114a</t>
         </is>
       </c>
-      <c r="D754" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E754" s="2" t="n"/>
-      <c r="F754" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Laptop Replacement Part - BA81-18114A</t>
-        </is>
-      </c>
-      <c r="G754" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H754" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D754" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E754" s="3" t="n"/>
+      <c r="F754" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Keyboard - BA81-18114A</t>
+        </is>
+      </c>
+      <c r="G754" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H754" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung BA81-18114A Keyboard|Samsung Parts USA | Keyboard / fits computer</t>
         </is>
       </c>
     </row>
@@ -30839,40 +30843,40 @@
       </c>
     </row>
     <row r="772">
-      <c r="A772" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B772" s="2" t="inlineStr">
+      <c r="A772" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B772" s="3" t="inlineStr">
         <is>
           <t>AH81-15423A</t>
         </is>
       </c>
-      <c r="C772" s="2" t="inlineStr">
+      <c r="C772" s="3" t="inlineStr">
         <is>
           <t>ah81-15423a</t>
         </is>
       </c>
-      <c r="D772" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E772" s="2" t="n"/>
-      <c r="F772" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH81-15423A</t>
-        </is>
-      </c>
-      <c r="G772" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H772" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D772" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E772" s="3" t="n"/>
+      <c r="F772" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Assembly Kit Main Service Jdm - AH81-15423A</t>
+        </is>
+      </c>
+      <c r="G772" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H772" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung samsung AH81-15423A SERVICE JDM-ASSEMBLY KIT MAIN|Samsung Parts USA | Service JDM-Assembly Kit Main / fits None</t>
         </is>
       </c>
     </row>
@@ -31113,40 +31117,40 @@
       </c>
     </row>
     <row r="779">
-      <c r="A779" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B779" s="2" t="inlineStr">
+      <c r="A779" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B779" s="3" t="inlineStr">
         <is>
           <t>AH94-03877B</t>
         </is>
       </c>
-      <c r="C779" s="2" t="inlineStr">
+      <c r="C779" s="3" t="inlineStr">
         <is>
           <t>ah94-03877b</t>
         </is>
       </c>
-      <c r="D779" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E779" s="2" t="n"/>
-      <c r="F779" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH94-03877B</t>
-        </is>
-      </c>
-      <c r="G779" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H779" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D779" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E779" s="3" t="n"/>
+      <c r="F779" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Assembly PCB Amp Rear Speaker-Right (Amp PCB Assembly) - AH94-03877B</t>
+        </is>
+      </c>
+      <c r="G779" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H779" s="3" t="inlineStr">
+        <is>
+          <t>Site title: samsung AH94-03877B ASSY PCB AMP REAR SPEAKER-RIGH– Samsung Parts USA | ASSY PCB AMP REAR SPEAKER-RIGHT (amp PCB assembly) / fits soundbar/speaker</t>
         </is>
       </c>
     </row>
@@ -32841,40 +32845,40 @@
       </c>
     </row>
     <row r="823">
-      <c r="A823" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B823" s="2" t="inlineStr">
+      <c r="A823" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B823" s="3" t="inlineStr">
         <is>
           <t>AH81-15425A</t>
         </is>
       </c>
-      <c r="C823" s="2" t="inlineStr">
+      <c r="C823" s="3" t="inlineStr">
         <is>
           <t>ah81-15425a</t>
         </is>
       </c>
-      <c r="D823" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E823" s="2" t="n"/>
-      <c r="F823" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH81-15425A</t>
-        </is>
-      </c>
-      <c r="G823" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H823" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D823" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E823" s="3" t="n"/>
+      <c r="F823" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Assembly Pba Main (Main Board) - AH81-15425A</t>
+        </is>
+      </c>
+      <c r="G823" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H823" s="3" t="inlineStr">
+        <is>
+          <t>Site title: samsung AH81-15425A ASSY PBA MAIN– Samsung Parts USA | ASSY PBA MAIN (main board) / fits soundbar/speaker</t>
         </is>
       </c>
     </row>
@@ -32959,40 +32963,40 @@
       </c>
     </row>
     <row r="826">
-      <c r="A826" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B826" s="2" t="inlineStr">
+      <c r="A826" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B826" s="3" t="inlineStr">
         <is>
           <t>AH82-01198A</t>
         </is>
       </c>
-      <c r="C826" s="2" t="inlineStr">
+      <c r="C826" s="3" t="inlineStr">
         <is>
           <t>ah82-01198a</t>
         </is>
       </c>
-      <c r="D826" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E826" s="2" t="n"/>
-      <c r="F826" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH82-01198A</t>
-        </is>
-      </c>
-      <c r="G826" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H826" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D826" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E826" s="3" t="n"/>
+      <c r="F826" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Assy-Speaker (Speaker Assembly) - AH82-01198A</t>
+        </is>
+      </c>
+      <c r="G826" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H826" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung AH82-01198A A/S ASSY-Speaker | A/S ASSY-Speaker (speaker assembly) / fits None</t>
         </is>
       </c>
     </row>
@@ -35613,40 +35617,40 @@
       </c>
     </row>
     <row r="893">
-      <c r="A893" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B893" s="2" t="inlineStr">
+      <c r="A893" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B893" s="3" t="inlineStr">
         <is>
           <t>6031-001531</t>
         </is>
       </c>
-      <c r="C893" s="2" t="inlineStr">
+      <c r="C893" s="3" t="inlineStr">
         <is>
           <t>6031-001531</t>
         </is>
       </c>
-      <c r="D893" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E893" s="2" t="n"/>
-      <c r="F893" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Replacement Part - 6031-001531</t>
-        </is>
-      </c>
-      <c r="G893" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H893" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D893" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E893" s="3" t="n"/>
+      <c r="F893" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Plain Washer - 6031-001531</t>
+        </is>
+      </c>
+      <c r="G893" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H893" s="3" t="inlineStr">
+        <is>
+          <t>Site title: 6031-001531 PLAIN WASHWER– Samsung Parts USA | Plain Washer / fits washing machine</t>
         </is>
       </c>
     </row>
@@ -36191,40 +36195,40 @@
       </c>
     </row>
     <row r="908">
-      <c r="A908" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B908" s="2" t="inlineStr">
+      <c r="A908" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B908" s="3" t="inlineStr">
         <is>
           <t>AH64-05867A</t>
         </is>
       </c>
-      <c r="C908" s="2" t="inlineStr">
+      <c r="C908" s="3" t="inlineStr">
         <is>
           <t>ah64-05867a</t>
         </is>
       </c>
-      <c r="D908" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E908" s="2" t="n"/>
-      <c r="F908" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH64-05867A</t>
-        </is>
-      </c>
-      <c r="G908" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H908" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D908" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E908" s="3" t="n"/>
+      <c r="F908" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Volume Button - AH64-05867A</t>
+        </is>
+      </c>
+      <c r="G908" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H908" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung AH64-05867A Button-Volume|Samsung Parts USA | Button-Volume / fits None</t>
         </is>
       </c>
     </row>
@@ -36869,78 +36873,78 @@
       </c>
     </row>
     <row r="925">
-      <c r="A925" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B925" s="2" t="inlineStr">
+      <c r="A925" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B925" s="3" t="inlineStr">
         <is>
           <t>AH81-11256A</t>
         </is>
       </c>
-      <c r="C925" s="2" t="inlineStr">
+      <c r="C925" s="3" t="inlineStr">
         <is>
           <t>ah81-11256a</t>
         </is>
       </c>
-      <c r="D925" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E925" s="2" t="n"/>
-      <c r="F925" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH81-11256A</t>
-        </is>
-      </c>
-      <c r="G925" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H925" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D925" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E925" s="3" t="n"/>
+      <c r="F925" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar DC Vss Power Board - AH81-11256A</t>
+        </is>
+      </c>
+      <c r="G925" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H925" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung AH81-11256A A/S-Dc Vss-Power Board– Samsung Parts USA | A/S-DC VSS Power Board / fits speaker/soundbar</t>
         </is>
       </c>
     </row>
     <row r="926">
-      <c r="A926" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B926" s="2" t="inlineStr">
+      <c r="A926" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B926" s="3" t="inlineStr">
         <is>
           <t>AH81-11262A</t>
         </is>
       </c>
-      <c r="C926" s="2" t="inlineStr">
+      <c r="C926" s="3" t="inlineStr">
         <is>
           <t>ah81-11262a</t>
         </is>
       </c>
-      <c r="D926" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E926" s="2" t="n"/>
-      <c r="F926" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH81-11262A</t>
-        </is>
-      </c>
-      <c r="G926" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H926" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D926" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E926" s="3" t="n"/>
+      <c r="F926" s="3" t="inlineStr">
+        <is>
+          <t>Samsung TV Speaker Right Assembly - AH81-11262A</t>
+        </is>
+      </c>
+      <c r="G926" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H926" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung AH81-11262A A/S-Assy-Speaker Right– Samsung Parts USA | A/S-Assy-Speaker Right / fits TV</t>
         </is>
       </c>
     </row>
@@ -37855,40 +37859,40 @@
       </c>
     </row>
     <row r="950">
-      <c r="A950" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B950" s="2" t="inlineStr">
+      <c r="A950" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B950" s="3" t="inlineStr">
         <is>
           <t>AH96-02267E</t>
         </is>
       </c>
-      <c r="C950" s="2" t="inlineStr">
+      <c r="C950" s="3" t="inlineStr">
         <is>
           <t>ah96-02267e</t>
         </is>
       </c>
-      <c r="D950" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E950" s="2" t="n"/>
-      <c r="F950" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH96-02267E</t>
-        </is>
-      </c>
-      <c r="G950" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H950" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D950" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E950" s="3" t="n"/>
+      <c r="F950" s="3" t="inlineStr">
+        <is>
+          <t>Samsung TV Deck Assembly - AH96-02267E</t>
+        </is>
+      </c>
+      <c r="G950" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H950" s="3" t="inlineStr">
+        <is>
+          <t>Site title: AH96-02267E Deck Assembly– Samsung Parts USA | Deck Assembly / fits TV</t>
         </is>
       </c>
     </row>
@@ -40675,40 +40679,40 @@
       </c>
     </row>
     <row r="1022">
-      <c r="A1022" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1022" s="2" t="inlineStr">
+      <c r="A1022" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1022" s="3" t="inlineStr">
         <is>
           <t>AH81-13844A</t>
         </is>
       </c>
-      <c r="C1022" s="2" t="inlineStr">
+      <c r="C1022" s="3" t="inlineStr">
         <is>
           <t>ah81-13844a</t>
         </is>
       </c>
-      <c r="D1022" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1022" s="2" t="n"/>
-      <c r="F1022" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH81-13844A</t>
-        </is>
-      </c>
-      <c r="G1022" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1022" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1022" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1022" s="3" t="n"/>
+      <c r="F1022" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Wireless Audio Network - AH81-13844A</t>
+        </is>
+      </c>
+      <c r="G1022" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1022" s="3" t="inlineStr">
+        <is>
+          <t>Site title: samsung AH81-13844A A/S-NETWORK-WIRELESS AUDIO;WSA– Samsung Parts USA | A/S-Network-Wireless Audio;WSA / fits soundbar/speaker</t>
         </is>
       </c>
     </row>
@@ -41759,40 +41763,40 @@
       </c>
     </row>
     <row r="1050">
-      <c r="A1050" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1050" s="2" t="inlineStr">
+      <c r="A1050" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1050" s="3" t="inlineStr">
         <is>
           <t>BA98-02175A</t>
         </is>
       </c>
-      <c r="C1050" s="2" t="inlineStr">
+      <c r="C1050" s="3" t="inlineStr">
         <is>
           <t>ba98-02175a</t>
         </is>
       </c>
-      <c r="D1050" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1050" s="2" t="n"/>
-      <c r="F1050" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Laptop Replacement Part - BA98-02175A</t>
-        </is>
-      </c>
-      <c r="G1050" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1050" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1050" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1050" s="3" t="n"/>
+      <c r="F1050" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Top Case Front Assembly - BA98-02175A</t>
+        </is>
+      </c>
+      <c r="G1050" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1050" s="3" t="inlineStr">
+        <is>
+          <t>Site title: BA98-02175A ASSEMBLY CASE FRONT-TOP;JOAN-1– Samsung Parts USA | Assembly Case Front-Top / fits Chromebook (laptop)</t>
         </is>
       </c>
     </row>
@@ -42383,40 +42387,40 @@
       </c>
     </row>
     <row r="1066">
-      <c r="A1066" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1066" s="2" t="inlineStr">
+      <c r="A1066" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1066" s="3" t="inlineStr">
         <is>
           <t>AH81-11539A</t>
         </is>
       </c>
-      <c r="C1066" s="2" t="inlineStr">
+      <c r="C1066" s="3" t="inlineStr">
         <is>
           <t>ah81-11539a</t>
         </is>
       </c>
-      <c r="D1066" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1066" s="2" t="n"/>
-      <c r="F1066" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH81-11539A</t>
-        </is>
-      </c>
-      <c r="G1066" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1066" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1066" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1066" s="3" t="n"/>
+      <c r="F1066" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar La Panel - AH81-11539A</t>
+        </is>
+      </c>
+      <c r="G1066" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1066" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung AH81-11539A A/S-LA PANEL;08-0MXT70-LA0S,TO– Samsung Parts USA | A/S-LA Panel / fits soundbar/speaker</t>
         </is>
       </c>
     </row>
@@ -43015,40 +43019,40 @@
       </c>
     </row>
     <row r="1082">
-      <c r="A1082" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1082" s="2" t="inlineStr">
+      <c r="A1082" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1082" s="3" t="inlineStr">
         <is>
           <t>3601-001637</t>
         </is>
       </c>
-      <c r="C1082" s="2" t="inlineStr">
+      <c r="C1082" s="3" t="inlineStr">
         <is>
           <t>3601-001637</t>
         </is>
       </c>
-      <c r="D1082" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1082" s="2" t="n"/>
-      <c r="F1082" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Replacement Part - 3601-001637</t>
-        </is>
-      </c>
-      <c r="G1082" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1082" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1082" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1082" s="3" t="n"/>
+      <c r="F1082" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Range Cartridge Fuse - 3601-001637</t>
+        </is>
+      </c>
+      <c r="G1082" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1082" s="3" t="inlineStr">
+        <is>
+          <t>Site title: 3601-001637 FUSE-CARTRIDGE– Samsung Parts USA | Fuse-Cartridge / fits range/oven</t>
         </is>
       </c>
     </row>
@@ -44001,78 +44005,78 @@
       </c>
     </row>
     <row r="1107">
-      <c r="A1107" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1107" s="2" t="inlineStr">
+      <c r="A1107" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1107" s="3" t="inlineStr">
         <is>
           <t>4709-002533</t>
         </is>
       </c>
-      <c r="C1107" s="2" t="inlineStr">
+      <c r="C1107" s="3" t="inlineStr">
         <is>
           <t>4709-002533</t>
         </is>
       </c>
-      <c r="D1107" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1107" s="2" t="n"/>
-      <c r="F1107" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Replacement Part - 4709-002533</t>
-        </is>
-      </c>
-      <c r="G1107" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1107" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1107" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1107" s="3" t="n"/>
+      <c r="F1107" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Washer Lan Module W - 4709-002533</t>
+        </is>
+      </c>
+      <c r="G1107" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1107" s="3" t="inlineStr">
+        <is>
+          <t>Site title: 4709-002533 W-LAN MODULE– Samsung Parts USA | W-LAN Module / fits dishwasher</t>
         </is>
       </c>
     </row>
     <row r="1108">
-      <c r="A1108" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1108" s="2" t="inlineStr">
+      <c r="A1108" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1108" s="3" t="inlineStr">
         <is>
           <t>AH94-03807A</t>
         </is>
       </c>
-      <c r="C1108" s="2" t="inlineStr">
+      <c r="C1108" s="3" t="inlineStr">
         <is>
           <t>ah94-03807a</t>
         </is>
       </c>
-      <c r="D1108" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1108" s="2" t="n"/>
-      <c r="F1108" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH94-03807A</t>
-        </is>
-      </c>
-      <c r="G1108" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1108" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1108" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1108" s="3" t="n"/>
+      <c r="F1108" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar PCB Main Assembly - AH94-03807A</t>
+        </is>
+      </c>
+      <c r="G1108" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1108" s="3" t="inlineStr">
+        <is>
+          <t>Site title: AH94-03807A PCB Main Assembly– Samsung Parts USA | PCB Main Assembly / fits soundbar/TV (listing inconsistent)</t>
         </is>
       </c>
     </row>
@@ -44313,40 +44317,40 @@
       </c>
     </row>
     <row r="1115">
-      <c r="A1115" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1115" s="2" t="inlineStr">
+      <c r="A1115" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1115" s="3" t="inlineStr">
         <is>
           <t>AH81-15422A</t>
         </is>
       </c>
-      <c r="C1115" s="2" t="inlineStr">
+      <c r="C1115" s="3" t="inlineStr">
         <is>
           <t>ah81-15422a</t>
         </is>
       </c>
-      <c r="D1115" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1115" s="2" t="n"/>
-      <c r="F1115" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH81-15422A</t>
-        </is>
-      </c>
-      <c r="G1115" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1115" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1115" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1115" s="3" t="n"/>
+      <c r="F1115" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Assembly Spk Sub Service Jdm - AH81-15422A</t>
+        </is>
+      </c>
+      <c r="G1115" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1115" s="3" t="inlineStr">
+        <is>
+          <t>Site title: samsung AH81-15422A SERVICE JDM-ASSEMBLY SPK SUB– Samsung Parts USA | Service JDM-Assembly Spk Sub / fits speaker/soundbar</t>
         </is>
       </c>
     </row>
@@ -45863,78 +45867,78 @@
       </c>
     </row>
     <row r="1154">
-      <c r="A1154" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1154" s="2" t="inlineStr">
+      <c r="A1154" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1154" s="3" t="inlineStr">
         <is>
           <t>AH81-13713A</t>
         </is>
       </c>
-      <c r="C1154" s="2" t="inlineStr">
+      <c r="C1154" s="3" t="inlineStr">
         <is>
           <t>ah81-13713a</t>
         </is>
       </c>
-      <c r="D1154" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1154" s="2" t="n"/>
-      <c r="F1154" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH81-13713A</t>
-        </is>
-      </c>
-      <c r="G1154" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1154" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1154" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1154" s="3" t="n"/>
+      <c r="F1154" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Wl Wireless Module Service Jdm - AH81-13713A</t>
+        </is>
+      </c>
+      <c r="G1154" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1154" s="3" t="inlineStr">
+        <is>
+          <t>Site title: samsung AH81-13713A SERVICE JDM-WL WIRELESS MODULE– Samsung Parts USA | Service JDM-WL Wireless Module / fits None</t>
         </is>
       </c>
     </row>
     <row r="1155">
-      <c r="A1155" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1155" s="2" t="inlineStr">
+      <c r="A1155" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1155" s="3" t="inlineStr">
         <is>
           <t>AH81-14701A</t>
         </is>
       </c>
-      <c r="C1155" s="2" t="inlineStr">
+      <c r="C1155" s="3" t="inlineStr">
         <is>
           <t>ah81-14701a</t>
         </is>
       </c>
-      <c r="D1155" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1155" s="2" t="n"/>
-      <c r="F1155" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH81-14701A</t>
-        </is>
-      </c>
-      <c r="G1155" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1155" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1155" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1155" s="3" t="n"/>
+      <c r="F1155" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Service Jdm Pba-Main (Main PCB Assembly) - AH81-14701A</t>
+        </is>
+      </c>
+      <c r="G1155" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1155" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung AH81-14701A Svc Jdm Pba-Main|Samsung Parts USA | Svc Jdm Pba-Main (main PCB assembly) / fits None</t>
         </is>
       </c>
     </row>
@@ -47679,40 +47683,40 @@
       </c>
     </row>
     <row r="1200">
-      <c r="A1200" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1200" s="2" t="inlineStr">
+      <c r="A1200" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1200" s="3" t="inlineStr">
         <is>
           <t>AH83-00496A</t>
         </is>
       </c>
-      <c r="C1200" s="2" t="inlineStr">
+      <c r="C1200" s="3" t="inlineStr">
         <is>
           <t>ah83-00496a</t>
         </is>
       </c>
-      <c r="D1200" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1200" s="2" t="n"/>
-      <c r="F1200" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH83-00496A</t>
-        </is>
-      </c>
-      <c r="G1200" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1200" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1200" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1200" s="3" t="n"/>
+      <c r="F1200" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Speaker Wire Ckd - AH83-00496A</t>
+        </is>
+      </c>
+      <c r="G1200" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1200" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung samsung AH83-00496A CKD-SPEAKER WIRE|Samsung Parts USA | CKD-Speaker Wire / fits None</t>
         </is>
       </c>
     </row>
@@ -48623,40 +48627,40 @@
       </c>
     </row>
     <row r="1224">
-      <c r="A1224" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1224" s="2" t="inlineStr">
+      <c r="A1224" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1224" s="3" t="inlineStr">
         <is>
           <t>AH81-09744A</t>
         </is>
       </c>
-      <c r="C1224" s="2" t="inlineStr">
+      <c r="C1224" s="3" t="inlineStr">
         <is>
           <t>ah81-09744a</t>
         </is>
       </c>
-      <c r="D1224" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1224" s="2" t="n"/>
-      <c r="F1224" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH81-09744A</t>
-        </is>
-      </c>
-      <c r="G1224" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1224" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1224" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1224" s="3" t="n"/>
+      <c r="F1224" s="3" t="inlineStr">
+        <is>
+          <t>Samsung DC Vss Power Board - AH81-09744A</t>
+        </is>
+      </c>
+      <c r="G1224" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1224" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung AH81-09744A A/S-Dc Vss-Power Board;Tps2100|Samsung Parts USA | A/S-DC VSS Power Board / fits None</t>
         </is>
       </c>
     </row>
@@ -49681,40 +49685,40 @@
       </c>
     </row>
     <row r="1251">
-      <c r="A1251" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1251" s="2" t="inlineStr">
+      <c r="A1251" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1251" s="3" t="inlineStr">
         <is>
           <t>AH39-00540A</t>
         </is>
       </c>
-      <c r="C1251" s="2" t="inlineStr">
+      <c r="C1251" s="3" t="inlineStr">
         <is>
           <t>ah39-00540a</t>
         </is>
       </c>
-      <c r="D1251" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1251" s="2" t="n"/>
-      <c r="F1251" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH39-00540A</t>
-        </is>
-      </c>
-      <c r="G1251" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1251" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1251" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1251" s="3" t="n"/>
+      <c r="F1251" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Cable Interface - AH39-00540A</t>
+        </is>
+      </c>
+      <c r="G1251" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1251" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung AH39-00540A CBF INTERFACE|Samsung Parts USA | CBF Interface / fits None</t>
         </is>
       </c>
     </row>
@@ -51341,40 +51345,40 @@
       </c>
     </row>
     <row r="1293">
-      <c r="A1293" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1293" s="2" t="inlineStr">
+      <c r="A1293" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1293" s="3" t="inlineStr">
         <is>
           <t>4709-002892</t>
         </is>
       </c>
-      <c r="C1293" s="2" t="inlineStr">
+      <c r="C1293" s="3" t="inlineStr">
         <is>
           <t>4709-002892</t>
         </is>
       </c>
-      <c r="D1293" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1293" s="2" t="n"/>
-      <c r="F1293" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Replacement Part - 4709-002892</t>
-        </is>
-      </c>
-      <c r="G1293" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1293" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit (only 4709-002829)</t>
+      <c r="D1293" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1293" s="3" t="n"/>
+      <c r="F1293" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Refrigerator W Lan Module - 4709-002892</t>
+        </is>
+      </c>
+      <c r="G1293" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1293" s="3" t="inlineStr">
+        <is>
+          <t>Site title: 4709-002892 W Lan Module– Samsung Parts USA | W Lan Module / fits refrigerator</t>
         </is>
       </c>
     </row>
@@ -52129,40 +52133,40 @@
       </c>
     </row>
     <row r="1313">
-      <c r="A1313" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1313" s="2" t="inlineStr">
+      <c r="A1313" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1313" s="3" t="inlineStr">
         <is>
           <t>7UQ75-40028</t>
         </is>
       </c>
-      <c r="C1313" s="2" t="inlineStr">
+      <c r="C1313" s="3" t="inlineStr">
         <is>
           <t>7uq75-40028</t>
         </is>
       </c>
-      <c r="D1313" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1313" s="2" t="n"/>
-      <c r="F1313" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Replacement Part - 7UQ75-40028</t>
-        </is>
-      </c>
-      <c r="G1313" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1313" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1313" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1313" s="3" t="n"/>
+      <c r="F1313" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Cassette - 7UQ75-40028</t>
+        </is>
+      </c>
+      <c r="G1313" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1313" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung 7UQ75-40028 CASSETTE|Samsung Parts USA | Cassette / fits None</t>
         </is>
       </c>
     </row>
@@ -52327,40 +52331,40 @@
       </c>
     </row>
     <row r="1318">
-      <c r="A1318" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1318" s="2" t="inlineStr">
+      <c r="A1318" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1318" s="3" t="inlineStr">
         <is>
           <t>AH81-11487A</t>
         </is>
       </c>
-      <c r="C1318" s="2" t="inlineStr">
+      <c r="C1318" s="3" t="inlineStr">
         <is>
           <t>ah81-11487a</t>
         </is>
       </c>
-      <c r="D1318" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1318" s="2" t="n"/>
-      <c r="F1318" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Replacement Part - AH81-11487A</t>
-        </is>
-      </c>
-      <c r="G1318" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1318" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1318" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1318" s="3" t="n"/>
+      <c r="F1318" s="3" t="inlineStr">
+        <is>
+          <t>Samsung A S Aux Board - AH81-11487A</t>
+        </is>
+      </c>
+      <c r="G1318" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1318" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung AH81-11487A A S Aux Board|Samsung Parts USA | A S Aux Board / fits None</t>
         </is>
       </c>
     </row>
@@ -52521,40 +52525,40 @@
       </c>
     </row>
     <row r="1323">
-      <c r="A1323" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1323" s="2" t="inlineStr">
+      <c r="A1323" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1323" s="3" t="inlineStr">
         <is>
           <t>4712-001033</t>
         </is>
       </c>
-      <c r="C1323" s="2" t="inlineStr">
+      <c r="C1323" s="3" t="inlineStr">
         <is>
           <t>4712-001033</t>
         </is>
       </c>
-      <c r="D1323" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1323" s="2" t="n"/>
-      <c r="F1323" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Replacement Part - 4712-001033</t>
-        </is>
-      </c>
-      <c r="G1323" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1323" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1323" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1323" s="3" t="n"/>
+      <c r="F1323" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Thermostat - 4712-001033</t>
+        </is>
+      </c>
+      <c r="G1323" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1323" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung 4712-001033 Thermostat|Samsung Parts USA | Thermostat / fits None</t>
         </is>
       </c>
     </row>
@@ -54135,40 +54139,40 @@
       </c>
     </row>
     <row r="1364">
-      <c r="A1364" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1364" s="2" t="inlineStr">
+      <c r="A1364" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1364" s="3" t="inlineStr">
         <is>
           <t>AA59-00599A</t>
         </is>
       </c>
-      <c r="C1364" s="2" t="inlineStr">
+      <c r="C1364" s="3" t="inlineStr">
         <is>
           <t>aa59-00599a</t>
         </is>
       </c>
-      <c r="D1364" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1364" s="2" t="n"/>
-      <c r="F1364" s="2" t="inlineStr">
-        <is>
-          <t>Samsung AV Replacement Part - AA59-00599A</t>
-        </is>
-      </c>
-      <c r="G1364" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1364" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1364" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1364" s="3" t="n"/>
+      <c r="F1364" s="3" t="inlineStr">
+        <is>
+          <t>Samsung TV Remote Control - AA59-00599A</t>
+        </is>
+      </c>
+      <c r="G1364" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1364" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung AA59-00599A TV Remote Control|Samsung Parts USA | TV Remote Control / fits TV</t>
         </is>
       </c>
     </row>
@@ -57579,40 +57583,40 @@
       </c>
     </row>
     <row r="1452">
-      <c r="A1452" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1452" s="2" t="inlineStr">
+      <c r="A1452" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1452" s="3" t="inlineStr">
         <is>
           <t>3701-001905</t>
         </is>
       </c>
-      <c r="C1452" s="2" t="inlineStr">
+      <c r="C1452" s="3" t="inlineStr">
         <is>
           <t>3701-001905</t>
         </is>
       </c>
-      <c r="D1452" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1452" s="2" t="n"/>
-      <c r="F1452" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Replacement Part - 3701-001905</t>
-        </is>
-      </c>
-      <c r="G1452" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1452" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1452" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1452" s="3" t="n"/>
+      <c r="F1452" s="3" t="inlineStr">
+        <is>
+          <t>Samsung HDMI Connector - 3701-001905</t>
+        </is>
+      </c>
+      <c r="G1452" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1452" s="3" t="inlineStr">
+        <is>
+          <t>Site title: 3701-001905 CONNECTOR-HDMI– Samsung Parts USA | Connector-HDMI / fits None</t>
         </is>
       </c>
     </row>
@@ -58009,40 +58013,40 @@
       </c>
     </row>
     <row r="1463">
-      <c r="A1463" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1463" s="2" t="inlineStr">
+      <c r="A1463" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1463" s="3" t="inlineStr">
         <is>
           <t>3001-002842</t>
         </is>
       </c>
-      <c r="C1463" s="2" t="inlineStr">
+      <c r="C1463" s="3" t="inlineStr">
         <is>
           <t>3001-002842</t>
         </is>
       </c>
-      <c r="D1463" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1463" s="2" t="n"/>
-      <c r="F1463" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Replacement Part - 3001-002842</t>
-        </is>
-      </c>
-      <c r="G1463" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1463" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1463" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1463" s="3" t="n"/>
+      <c r="F1463" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Refrigerator Speaker - 3001-002842</t>
+        </is>
+      </c>
+      <c r="G1463" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1463" s="3" t="inlineStr">
+        <is>
+          <t>Site title: 3001-002842 SPEAKER– Samsung Parts USA | Speaker / fits refrigerator</t>
         </is>
       </c>
     </row>
@@ -59631,40 +59635,40 @@
       </c>
     </row>
     <row r="1504">
-      <c r="A1504" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1504" s="2" t="inlineStr">
+      <c r="A1504" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1504" s="3" t="inlineStr">
         <is>
           <t>3708-003073</t>
         </is>
       </c>
-      <c r="C1504" s="2" t="inlineStr">
+      <c r="C1504" s="3" t="inlineStr">
         <is>
           <t>3708-003073</t>
         </is>
       </c>
-      <c r="D1504" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1504" s="2" t="n"/>
-      <c r="F1504" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Replacement Part - 3708-003073</t>
-        </is>
-      </c>
-      <c r="G1504" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1504" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1504" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1504" s="3" t="n"/>
+      <c r="F1504" s="3" t="inlineStr">
+        <is>
+          <t>Samsung TV Connector-Fpc/Ffc/Pic - 3708-003073</t>
+        </is>
+      </c>
+      <c r="G1504" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1504" s="3" t="inlineStr">
+        <is>
+          <t>Site title: 3708-003073 CONNECTOR-FPC/FFC/PIC– Samsung Parts USA | Connector-FPC/FFC/PIC / fits TV</t>
         </is>
       </c>
     </row>
@@ -59909,40 +59913,40 @@
       </c>
     </row>
     <row r="1511">
-      <c r="A1511" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1511" s="2" t="inlineStr">
+      <c r="A1511" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1511" s="3" t="inlineStr">
         <is>
           <t>3705-001191</t>
         </is>
       </c>
-      <c r="C1511" s="2" t="inlineStr">
+      <c r="C1511" s="3" t="inlineStr">
         <is>
           <t>3705-001191</t>
         </is>
       </c>
-      <c r="D1511" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1511" s="2" t="n"/>
-      <c r="F1511" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Replacement Part - 3705-001191</t>
-        </is>
-      </c>
-      <c r="G1511" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1511" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1511" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1511" s="3" t="n"/>
+      <c r="F1511" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Coaxial Connector - 3705-001191</t>
+        </is>
+      </c>
+      <c r="G1511" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1511" s="3" t="inlineStr">
+        <is>
+          <t>Site title: 3705-001191 CONNECTOR-COAXIAL– Samsung Parts USA | Connector-Coaxial / fits None</t>
         </is>
       </c>
     </row>
@@ -61025,40 +61029,40 @@
       </c>
     </row>
     <row r="1539">
-      <c r="A1539" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1539" s="2" t="inlineStr">
+      <c r="A1539" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1539" s="3" t="inlineStr">
         <is>
           <t>1205-006618</t>
         </is>
       </c>
-      <c r="C1539" s="2" t="inlineStr">
+      <c r="C1539" s="3" t="inlineStr">
         <is>
           <t>1205-006618</t>
         </is>
       </c>
-      <c r="D1539" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1539" s="2" t="n"/>
-      <c r="F1539" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Replacement Part - 1205-006618</t>
-        </is>
-      </c>
-      <c r="G1539" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1539" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1539" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1539" s="3" t="n"/>
+      <c r="F1539" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Ic-Nfc/Rfid - 1205-006618</t>
+        </is>
+      </c>
+      <c r="G1539" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1539" s="3" t="inlineStr">
+        <is>
+          <t>Site title: Samsung 1205-006618 Ic-Nfc/Rfid;Sn220Uuk/B026C0,3.– Samsung Parts USA | IC-NFC/RFID / fits None</t>
         </is>
       </c>
     </row>
@@ -61299,40 +61303,40 @@
       </c>
     </row>
     <row r="1546">
-      <c r="A1546" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B1546" s="2" t="inlineStr">
+      <c r="A1546" s="3" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B1546" s="3" t="inlineStr">
         <is>
           <t>0402-001195</t>
         </is>
       </c>
-      <c r="C1546" s="2" t="inlineStr">
+      <c r="C1546" s="3" t="inlineStr">
         <is>
           <t>0402-001195</t>
         </is>
       </c>
-      <c r="D1546" s="2" t="inlineStr">
-        <is>
-          <t>Predicted (page not found by search)</t>
-        </is>
-      </c>
-      <c r="E1546" s="2" t="n"/>
-      <c r="F1546" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Replacement Part - 0402-001195</t>
-        </is>
-      </c>
-      <c r="G1546" s="2" t="inlineStr">
-        <is>
-          <t>Placeholder</t>
-        </is>
-      </c>
-      <c r="H1546" s="2" t="inlineStr">
-        <is>
-          <t>PLACEHOLDER: part type not identified; brand/category guessed from part-number prefix only. Replace when a description is available. | searched, no exact hit</t>
+      <c r="D1546" s="3" t="inlineStr">
+        <is>
+          <t>Predicted (found only on another site)</t>
+        </is>
+      </c>
+      <c r="E1546" s="3" t="n"/>
+      <c r="F1546" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Rectifier Diode - 0402-001195</t>
+        </is>
+      </c>
+      <c r="G1546" s="3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H1546" s="3" t="inlineStr">
+        <is>
+          <t>Site title: 0402-001195 Diode-Rectifier, F1T4, 40– Samsung Parts USA | Diode-Rectifier / fits DVD player</t>
         </is>
       </c>
     </row>

</xml_diff>